<commit_message>
Add PMO timeline and dashboard visualizations
</commit_message>
<xml_diff>
--- a/data/project_tasks.xlsx
+++ b/data/project_tasks.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mauro\Documents\Portfolio PMO\PMO project dashboard\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mauro\Documents\Portfolio PMO\PMO-Project-Dashboard\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -137,9 +137,6 @@
     <t>T009</t>
   </si>
   <si>
-    <t>Go-Live</t>
-  </si>
-  <si>
     <t>Project Team</t>
   </si>
   <si>
@@ -147,6 +144,9 @@
   </si>
   <si>
     <t>Hypercare Support</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Go-Live </t>
   </si>
 </sst>
 </file>
@@ -756,10 +756,10 @@
         <v>5</v>
       </c>
       <c r="C10" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>37</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>38</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>29</v>
@@ -768,7 +768,7 @@
         <v>46143</v>
       </c>
       <c r="G10" s="3">
-        <v>46143</v>
+        <v>46145</v>
       </c>
       <c r="H10" s="2">
         <v>0</v>
@@ -779,13 +779,13 @@
     </row>
     <row r="11" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B11" s="2">
         <v>5</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>11</v>

</xml_diff>